<commit_message>
feat(clinical-knowledge): add orientation presentation targets
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{783FE0CA-EBFB-4F0B-B0F9-928245ED64EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE91FA9-9384-4389-9257-325B37F886D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13890" yWindow="165" windowWidth="11205" windowHeight="14865" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11220" yWindow="165" windowWidth="13875" windowHeight="14865" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10737" uniqueCount="2004">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10740" uniqueCount="2007">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6049,6 +6049,15 @@
   </si>
   <si>
     <t>functionalFacets</t>
+  </si>
+  <si>
+    <t>orientation.rehabilitation</t>
+  </si>
+  <si>
+    <t>orientation.apa</t>
+  </si>
+  <si>
+    <t>orientation.ordinaryAP</t>
   </si>
 </sst>
 </file>
@@ -54635,7 +54644,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -54858,6 +54867,19 @@
       <c r="E9" t="s">
         <v>1930</v>
       </c>
+      <c r="I9" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="I10" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="I11" t="s">
+        <v>2006</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(orientation): route rehabilitation guidance to Q1
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE91FA9-9384-4389-9257-325B37F886D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862FDE04-BC09-4628-AB4A-188B2CC09117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11220" yWindow="165" windowWidth="13875" windowHeight="14865" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11625" yWindow="630" windowWidth="13665" windowHeight="14865" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -6064,7 +6064,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -6086,8 +6086,13 @@
       <sz val="11"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6104,8 +6109,14 @@
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -6113,11 +6124,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6163,6 +6187,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7239,7 +7266,7 @@
         <v>162</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="37" spans="1:2">
@@ -7358,8 +7385,8 @@
       <c r="A51" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>403</v>
+      <c r="B51" s="12" t="s">
+        <v>2004</v>
       </c>
     </row>
     <row r="52" spans="1:2">
@@ -7374,8 +7401,8 @@
       <c r="A53" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>403</v>
+      <c r="B53" s="12" t="s">
+        <v>2004</v>
       </c>
     </row>
     <row r="54" spans="1:2">
@@ -7919,7 +7946,7 @@
         <v>727</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="28.5">
@@ -8207,7 +8234,7 @@
         <v>875</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="158" spans="1:2">
@@ -8295,7 +8322,7 @@
         <v>904</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="169" spans="1:2">
@@ -8719,7 +8746,7 @@
         <v>1131</v>
       </c>
       <c r="B221" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="222" spans="1:2" ht="28.5">
@@ -9031,7 +9058,7 @@
         <v>1280</v>
       </c>
       <c r="B260" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="261" spans="1:2">
@@ -9590,8 +9617,8 @@
       <c r="A330" s="2" t="s">
         <v>1567</v>
       </c>
-      <c r="B330" s="2" t="s">
-        <v>403</v>
+      <c r="B330" s="12" t="s">
+        <v>2004</v>
       </c>
     </row>
     <row r="331" spans="1:2">
@@ -10239,7 +10266,7 @@
         <v>1878</v>
       </c>
       <c r="B411" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="412" spans="1:2" ht="28.5">
@@ -10271,7 +10298,7 @@
         <v>1888</v>
       </c>
       <c r="B415" s="2" t="s">
-        <v>403</v>
+        <v>2004</v>
       </c>
     </row>
     <row r="416" spans="1:2" ht="28.5">
@@ -10340,17 +10367,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0900-000000000000}">
           <x14:formula1>
             <xm:f>Lists!$I$2:$I$8</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B423</xm:sqref>
+          <xm:sqref>B416:B423 B158:B259 B54:B156 B2:B35 B37:B50 B52 B261:B329 B331:B414</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" xr:uid="{42BFBFD1-A5F7-4BEE-9C24-9A47F33C1DE2}">
+          <x14:formula1>
+            <xm:f>Lists!$I$2:$I$11</xm:f>
+          </x14:formula1>
+          <xm:sqref>B36 B51 B53 B330</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
feat(orientation): classify APA benefit factors in clinical knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{862FDE04-BC09-4628-AB4A-188B2CC09117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70F9B3D-36BD-417F-BDA1-5D22D869C994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11625" yWindow="630" windowWidth="13665" windowHeight="14865" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13095" yWindow="270" windowWidth="15150" windowHeight="14865" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10740" uniqueCount="2007">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10740" uniqueCount="2008">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6058,6 +6058,9 @@
   </si>
   <si>
     <t>orientation.ordinaryAP</t>
+  </si>
+  <si>
+    <t>apaBenefitFactor</t>
   </si>
 </sst>
 </file>
@@ -6182,14 +6185,14 @@
         </x:ext>
       </extLst>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6507,16 +6510,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1">
       <c r="A2" s="2"/>
@@ -7385,7 +7388,7 @@
       <c r="A51" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="10" t="s">
         <v>2004</v>
       </c>
     </row>
@@ -7401,7 +7404,7 @@
       <c r="A53" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B53" s="10" t="s">
         <v>2004</v>
       </c>
     </row>
@@ -8402,7 +8405,7 @@
         <v>956</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>403</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="179" spans="1:2">
@@ -9298,7 +9301,7 @@
         <v>1395</v>
       </c>
       <c r="B290" s="2" t="s">
-        <v>403</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="291" spans="1:2">
@@ -9418,7 +9421,7 @@
         <v>1461</v>
       </c>
       <c r="B305" s="2" t="s">
-        <v>403</v>
+        <v>2005</v>
       </c>
     </row>
     <row r="306" spans="1:2">
@@ -9617,7 +9620,7 @@
       <c r="A330" s="2" t="s">
         <v>1567</v>
       </c>
-      <c r="B330" s="12" t="s">
+      <c r="B330" s="10" t="s">
         <v>2004</v>
       </c>
     </row>
@@ -32635,7 +32638,7 @@
         <v>232</v>
       </c>
       <c r="C234" t="s">
-        <v>395</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="235" spans="1:3">
@@ -34010,7 +34013,7 @@
         <v>232</v>
       </c>
       <c r="C359" t="s">
-        <v>395</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="360" spans="1:3">
@@ -34208,7 +34211,7 @@
         <v>232</v>
       </c>
       <c r="C377" t="s">
-        <v>395</v>
+        <v>2007</v>
       </c>
     </row>
     <row r="378" spans="1:3">

</xml_diff>

<commit_message>
Orientation C2 - integrate AOMI and HTA knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70F9B3D-36BD-417F-BDA1-5D22D869C994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD07A064-49E2-4DE3-B403-D98270274387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13095" yWindow="270" windowWidth="15150" windowHeight="14865" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10740" uniqueCount="2008">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10793" uniqueCount="2024">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6061,6 +6061,54 @@
   </si>
   <si>
     <t>apaBenefitFactor</t>
+  </si>
+  <si>
+    <t>aomi-orientation-vascular-rehabilitation-claudication-001</t>
+  </si>
+  <si>
+    <t>En cas d’AOMI avec claudication intermittente, la HAS recommande une réadaptation vasculaire en première intention. Examiner l’accès à un programme supervisé ou, en cas d’impossibilité, à une réadaptation structurée avec accompagnement. Claudication et modalités de prise en charge à vérifier.</t>
+  </si>
+  <si>
+    <t>Claudication intermittente, stabilité clinique, possibilités de réadaptation et avis spécialisé à apprécier par le médecin</t>
+  </si>
+  <si>
+    <t>C1 pilote. Message Q1 spécifique ; condition clinique non calculée. Sources HAS 2022 + fiche réadaptation 2024.</t>
+  </si>
+  <si>
+    <t>aomi-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>La HAS recommande un programme APA dans l’AOMI. En présence d’une claudication, distinguer le programme APA de la réadaptation vasculaire initiale et examiner les possibilités d’accompagnement ou de relais selon la situation du patient.</t>
+  </si>
+  <si>
+    <t>Présence de claudication, phase et besoin de réadaptation non déduits de la seule AOMI cochée</t>
+  </si>
+  <si>
+    <t>C1 pilote. Mention APA documentaire ; ne sélectionne pas automatiquement un niveau 2.</t>
+  </si>
+  <si>
+    <t>hta-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Chez les patients hypertendus, une activité physique régulière est recommandée. La synthèse HAS de 2022 propose également un programme APA supervisé ; son intérêt est à apprécier selon les besoins d’accompagnement, sans exclure une pratique autonome ou en sport-santé.</t>
+  </si>
+  <si>
+    <t>Équilibre de l’HTA, RCV, comorbidités, pratique antérieure et besoins d’accompagnement à apprécier</t>
+  </si>
+  <si>
+    <t>C1 pilote. Nuance HAS synthèse 2022 / référentiel 2018 ; pas d'indication automatique de niveau 2.</t>
+  </si>
+  <si>
+    <t>has-aps-aomi-07-2022</t>
+  </si>
+  <si>
+    <t>has-orientation-aomi-rehabilitation-10-2024</t>
+  </si>
+  <si>
+    <t>has-aps-hta-07-2022</t>
+  </si>
+  <si>
+    <t>has-ref-aps-hta-09-2018</t>
   </si>
 </sst>
 </file>
@@ -6312,7 +6360,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B6">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -6977,7 +7025,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B423"/>
+  <dimension ref="A1:B426"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -7481,12 +7529,8 @@
       </c>
     </row>
     <row r="63" spans="1:2">
-      <c r="A63" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>403</v>
-      </c>
+      <c r="A63" s="2"/>
+      <c r="B63" s="2"/>
     </row>
     <row r="64" spans="1:2">
       <c r="A64" s="2" t="s">
@@ -10366,6 +10410,30 @@
       </c>
       <c r="B423" s="2" t="s">
         <v>192</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2">
+      <c r="A424" s="8" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B424" s="8" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2">
+      <c r="A425" s="8" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B425" s="8" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2">
+      <c r="A426" s="8" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B426" s="8" t="s">
+        <v>2005</v>
       </c>
     </row>
   </sheetData>
@@ -10754,7 +10822,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D530"/>
+  <dimension ref="A1:D533"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -10989,16 +11057,10 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="28.5">
-      <c r="A19" s="8" t="s">
-        <v>336</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>403</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>1968</v>
-      </c>
+    <row r="19" spans="1:4">
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
       <c r="D19" s="8"/>
     </row>
     <row r="20" spans="1:4">
@@ -17304,6 +17366,39 @@
         <v>1979</v>
       </c>
       <c r="D530" s="8"/>
+    </row>
+    <row r="531" spans="1:4">
+      <c r="A531" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B531" t="s">
+        <v>403</v>
+      </c>
+      <c r="C531" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="532" spans="1:4">
+      <c r="A532" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B532" t="s">
+        <v>403</v>
+      </c>
+      <c r="C532" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="533" spans="1:4">
+      <c r="A533" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B533" t="s">
+        <v>403</v>
+      </c>
+      <c r="C533" t="s">
+        <v>1968</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17312,7 +17407,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I504"/>
+  <dimension ref="A1:I507"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -19433,8 +19528,8 @@
       <c r="F88" s="3" t="b">
         <v>0</v>
       </c>
-      <c r="G88" s="2" t="s">
-        <v>41</v>
+      <c r="G88" t="s">
+        <v>231</v>
       </c>
       <c r="H88" s="2">
         <v>1</v>
@@ -30037,6 +30132,84 @@
       </c>
       <c r="I504" s="2" t="s">
         <v>1914</v>
+      </c>
+    </row>
+    <row r="505" spans="1:9">
+      <c r="A505" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B505" t="s">
+        <v>2009</v>
+      </c>
+      <c r="D505" t="s">
+        <v>55</v>
+      </c>
+      <c r="E505" t="s">
+        <v>2010</v>
+      </c>
+      <c r="F505" t="b">
+        <v>0</v>
+      </c>
+      <c r="G505" t="s">
+        <v>41</v>
+      </c>
+      <c r="H505">
+        <v>1</v>
+      </c>
+      <c r="I505" t="s">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="506" spans="1:9">
+      <c r="A506" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B506" t="s">
+        <v>2013</v>
+      </c>
+      <c r="D506" t="s">
+        <v>55</v>
+      </c>
+      <c r="E506" t="s">
+        <v>2014</v>
+      </c>
+      <c r="F506" t="b">
+        <v>0</v>
+      </c>
+      <c r="G506" t="s">
+        <v>41</v>
+      </c>
+      <c r="H506">
+        <v>1</v>
+      </c>
+      <c r="I506" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="507" spans="1:9">
+      <c r="A507" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B507" t="s">
+        <v>2017</v>
+      </c>
+      <c r="D507" t="s">
+        <v>55</v>
+      </c>
+      <c r="E507" t="s">
+        <v>2018</v>
+      </c>
+      <c r="F507" t="b">
+        <v>0</v>
+      </c>
+      <c r="G507" t="s">
+        <v>41</v>
+      </c>
+      <c r="H507">
+        <v>1</v>
+      </c>
+      <c r="I507" t="s">
+        <v>2019</v>
       </c>
     </row>
   </sheetData>
@@ -30060,7 +30233,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C507"/>
+  <dimension ref="A1:C510"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -35642,6 +35815,39 @@
       </c>
       <c r="C507" t="s">
         <v>193</v>
+      </c>
+    </row>
+    <row r="508" spans="1:3">
+      <c r="A508" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B508" t="s">
+        <v>232</v>
+      </c>
+      <c r="C508" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="509" spans="1:3">
+      <c r="A509" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B509" t="s">
+        <v>232</v>
+      </c>
+      <c r="C509" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="510" spans="1:3">
+      <c r="A510" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B510" t="s">
+        <v>232</v>
+      </c>
+      <c r="C510" t="s">
+        <v>2007</v>
       </c>
     </row>
   </sheetData>
@@ -35659,7 +35865,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I504"/>
+  <dimension ref="A1:I507"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -43036,6 +43242,30 @@
       <c r="G504" s="2"/>
       <c r="H504" s="2"/>
       <c r="I504" s="2"/>
+    </row>
+    <row r="505" spans="1:9">
+      <c r="A505" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B505" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="506" spans="1:9">
+      <c r="A506" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B506" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="507" spans="1:9">
+      <c r="A507" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B507" t="s">
+        <v>205</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51191,7 +51421,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -51203,6 +51433,46 @@
       </c>
       <c r="B1" s="1" t="s">
         <v>217</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>2012</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>2016</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation C3.1 - add five HAS APA markers
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD07A064-49E2-4DE3-B403-D98270274387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A8E910-6B05-4568-ADE1-EE068531DD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11655" yWindow="165" windowWidth="13545" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10793" uniqueCount="2024">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10888" uniqueCount="2045">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6109,6 +6109,69 @@
   </si>
   <si>
     <t>has-ref-aps-hta-09-2018</t>
+  </si>
+  <si>
+    <t>dt1-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Dans le diabète de type 1, la HAS propose un programme d’activité physique adaptée, en articulation avec l’éducation thérapeutique et le suivi diabétologique. Examiner les besoins d’encadrement et les adaptations liées notamment au risque d’hypoglycémie.</t>
+  </si>
+  <si>
+    <t>Education thérapeutique spécialisée, adaptation insulinothérapie/risques hypo, suivi diabétologue</t>
+  </si>
+  <si>
+    <t>C3.1 — repère HAS Q2a ; la décision d’un programme supervisé n’est pas déduite du seul diagnostic. Regroupement UX transversal ultérieur.</t>
+  </si>
+  <si>
+    <t>dt2-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Dans le diabète de type 2, la HAS recommande un programme d’activité physique adaptée. Le parcours HAS envisage une réalisation encadrée ou autonome : apprécier les besoins spécifiques de supervision et les complications éventuelles avant de discuter le niveau 2.</t>
+  </si>
+  <si>
+    <t>Activité initiale insuffisante, complications, capacités, besoin d’encadrement</t>
+  </si>
+  <si>
+    <t>obesite-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>En cas de surpoids ou d’obésité, la HAS recommande un programme d’activité physique adaptée. Examiner l’inactivité, le déconditionnement, les douleurs et les besoins d’accompagnement ; le diagnostic ou l’IMC seul ne détermine pas le niveau de supervision.</t>
+  </si>
+  <si>
+    <t>Surpoids/obésité, déconditionnement, douleurs des articulations en charge, besoin d’accompagnement</t>
+  </si>
+  <si>
+    <t>asthme-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Dans l’asthme, la HAS propose un programme d’activité physique adaptée. Examiner le contrôle de la maladie, la prévention des symptômes à l’effort et les besoins réels d’encadrement ; un asthme contrôlé ne justifie pas automatiquement le niveau 2.</t>
+  </si>
+  <si>
+    <t>Contrôle asthme, prévention bronchoconstriction d’effort, AP actuelle et souhaitée</t>
+  </si>
+  <si>
+    <t>grossesse-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Pendant la grossesse, la HAS propose un programme d’activité physique adaptée. Vérifier les contre-indications médicales ou obstétricales et adapter la pratique ; une grossesse non compliquée n’implique pas automatiquement un programme supervisé de niveau 2.</t>
+  </si>
+  <si>
+    <t>Exclure CI obstétricales/médicales, personnaliser intensité selon trimestre et forme</t>
+  </si>
+  <si>
+    <t>has-aps-dt1-07-2022</t>
+  </si>
+  <si>
+    <t>has-parcours-dt2-07-2025</t>
+  </si>
+  <si>
+    <t>has-aps-surpoids-obesite-07-2022</t>
+  </si>
+  <si>
+    <t>has-aps-asthme-07-2022</t>
+  </si>
+  <si>
+    <t>has-aps-grossesse-07-2022</t>
   </si>
 </sst>
 </file>
@@ -6360,7 +6423,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B11">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7025,7 +7088,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B426"/>
+  <dimension ref="A1:B431"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10433,6 +10496,46 @@
         <v>2016</v>
       </c>
       <c r="B426" s="8" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2">
+      <c r="A427" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B427" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2">
+      <c r="A428" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B428" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2">
+      <c r="A429" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B429" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B430" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="431" spans="1:2">
+      <c r="A431" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B431" t="s">
         <v>2005</v>
       </c>
     </row>
@@ -10822,7 +10925,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D533"/>
+  <dimension ref="A1:D538"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17400,6 +17503,61 @@
         <v>1968</v>
       </c>
     </row>
+    <row r="534" spans="1:4">
+      <c r="A534" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B534" t="s">
+        <v>403</v>
+      </c>
+      <c r="C534" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="535" spans="1:4">
+      <c r="A535" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B535" t="s">
+        <v>403</v>
+      </c>
+      <c r="C535" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="536" spans="1:4">
+      <c r="A536" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B536" t="s">
+        <v>403</v>
+      </c>
+      <c r="C536" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="537" spans="1:4">
+      <c r="A537" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B537" t="s">
+        <v>403</v>
+      </c>
+      <c r="C537" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="538" spans="1:4">
+      <c r="A538" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B538" t="s">
+        <v>403</v>
+      </c>
+      <c r="C538" t="s">
+        <v>1968</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17407,7 +17565,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I507"/>
+  <dimension ref="A1:I512"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30210,6 +30368,136 @@
       </c>
       <c r="I507" t="s">
         <v>2019</v>
+      </c>
+    </row>
+    <row r="508" spans="1:9">
+      <c r="A508" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B508" t="s">
+        <v>2025</v>
+      </c>
+      <c r="D508" t="s">
+        <v>55</v>
+      </c>
+      <c r="E508" t="s">
+        <v>2026</v>
+      </c>
+      <c r="F508" t="s">
+        <v>40</v>
+      </c>
+      <c r="G508" t="s">
+        <v>41</v>
+      </c>
+      <c r="H508">
+        <v>1</v>
+      </c>
+      <c r="I508" t="s">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="509" spans="1:9">
+      <c r="A509" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B509" t="s">
+        <v>2029</v>
+      </c>
+      <c r="D509" t="s">
+        <v>55</v>
+      </c>
+      <c r="E509" t="s">
+        <v>2030</v>
+      </c>
+      <c r="F509" t="s">
+        <v>40</v>
+      </c>
+      <c r="G509" t="s">
+        <v>41</v>
+      </c>
+      <c r="H509">
+        <v>1</v>
+      </c>
+      <c r="I509" t="s">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="510" spans="1:9">
+      <c r="A510" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B510" t="s">
+        <v>2032</v>
+      </c>
+      <c r="D510" t="s">
+        <v>55</v>
+      </c>
+      <c r="E510" t="s">
+        <v>2033</v>
+      </c>
+      <c r="F510" t="s">
+        <v>40</v>
+      </c>
+      <c r="G510" t="s">
+        <v>41</v>
+      </c>
+      <c r="H510">
+        <v>1</v>
+      </c>
+      <c r="I510" t="s">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="511" spans="1:9">
+      <c r="A511" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B511" t="s">
+        <v>2035</v>
+      </c>
+      <c r="D511" t="s">
+        <v>55</v>
+      </c>
+      <c r="E511" t="s">
+        <v>2036</v>
+      </c>
+      <c r="F511" t="s">
+        <v>40</v>
+      </c>
+      <c r="G511" t="s">
+        <v>41</v>
+      </c>
+      <c r="H511">
+        <v>1</v>
+      </c>
+      <c r="I511" t="s">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="512" spans="1:9">
+      <c r="A512" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B512" t="s">
+        <v>2038</v>
+      </c>
+      <c r="D512" t="s">
+        <v>55</v>
+      </c>
+      <c r="E512" t="s">
+        <v>2039</v>
+      </c>
+      <c r="F512" t="s">
+        <v>40</v>
+      </c>
+      <c r="G512" t="s">
+        <v>41</v>
+      </c>
+      <c r="H512">
+        <v>1</v>
+      </c>
+      <c r="I512" t="s">
+        <v>2027</v>
       </c>
     </row>
   </sheetData>
@@ -30233,7 +30521,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C510"/>
+  <dimension ref="A1:C515"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -35847,6 +36135,61 @@
         <v>232</v>
       </c>
       <c r="C510" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="511" spans="1:3">
+      <c r="A511" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B511" t="s">
+        <v>232</v>
+      </c>
+      <c r="C511" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="512" spans="1:3">
+      <c r="A512" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B512" t="s">
+        <v>232</v>
+      </c>
+      <c r="C512" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="513" spans="1:3">
+      <c r="A513" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B513" t="s">
+        <v>232</v>
+      </c>
+      <c r="C513" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="514" spans="1:3">
+      <c r="A514" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B514" t="s">
+        <v>232</v>
+      </c>
+      <c r="C514" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="515" spans="1:3">
+      <c r="A515" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B515" t="s">
+        <v>232</v>
+      </c>
+      <c r="C515" t="s">
         <v>2007</v>
       </c>
     </row>
@@ -35865,7 +36208,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I507"/>
+  <dimension ref="A1:I512"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -43265,6 +43608,46 @@
       </c>
       <c r="B507" t="s">
         <v>205</v>
+      </c>
+    </row>
+    <row r="508" spans="1:9">
+      <c r="A508" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B508" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="509" spans="1:9">
+      <c r="A509" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B509" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="510" spans="1:9">
+      <c r="A510" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B510" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="511" spans="1:9">
+      <c r="A511" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B511" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="512" spans="1:9">
+      <c r="A512" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B512" t="s">
+        <v>1796</v>
       </c>
     </row>
   </sheetData>
@@ -51421,7 +51804,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -51473,6 +51856,46 @@
       </c>
       <c r="B6" t="s">
         <v>2023</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>2024</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>2028</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2041</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>2031</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2042</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>2034</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>2037</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation C3.2 - add four specific APA guidance items
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A8E910-6B05-4568-ADE1-EE068531DD75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21EF102-5997-4029-876D-2FA85E6E6606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11655" yWindow="165" windowWidth="13545" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10888" uniqueCount="2045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10964" uniqueCount="2062">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6172,6 +6172,57 @@
   </si>
   <si>
     <t>has-aps-grossesse-07-2022</t>
+  </si>
+  <si>
+    <t>coronaropathie-orientation-apa-post-rehabilitation-001</t>
+  </si>
+  <si>
+    <t>Pour une coronaropathie, vérifier si une réadaptation cardiovasculaire est indiquée ou a été réalisée. Au décours, la HAS prévoit un programme d’APA appuyé sur le bilan et les consignes de sortie ; selon le risque, les capacités et l’autonomie, cette poursuite peut être supervisée ou autonome. Ne pas en déduire systématiquement un niveau 2.</t>
+  </si>
+  <si>
+    <t>Contexte coronarien stable ou après événement aigu, réadaptation réalisée/indiquée, bilan et consignes de sortie à vérifier.</t>
+  </si>
+  <si>
+    <t>C3.2 — complément Q2a spécifique : repère conditionnel ; aucune orientation automatique ni usage Q1 modifié.</t>
+  </si>
+  <si>
+    <t>icc-orientation-apa-post-rehabilitation-001</t>
+  </si>
+  <si>
+    <t>Pour une insuffisance cardiaque chronique stable, examiner la réadaptation cardiovasculaire et, si elle a été réalisée, les consignes d’exercice à sa sortie. La HAS recommande une APA régulière ; l’accompagnement professionnel et les modalités de poursuite sont à apprécier selon symptômes, capacités, risques et autonomie, sans imposer automatiquement le niveau 2.</t>
+  </si>
+  <si>
+    <t>Stabilité et compensation de l'ICC, symptômes, réadaptation antérieure, bilan et plan de sortie non présumés.</t>
+  </si>
+  <si>
+    <t>bpco-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Dans une BPCO stabilisée, une activité physique adaptée régulière est utile. Si dyspnée, intolérance à l’effort ou limitation des activités malgré une prise en charge optimisée, examiner d’abord l’indication de réadaptation respiratoire ; un programme d’APA peut contribuer à la poursuite des acquis selon les capacités et les besoins d’encadrement. Une pratique autonome reste possible selon la situation.</t>
+  </si>
+  <si>
+    <t>Dyspnée/retentissement fonctionnel, exacerbations, traitement optimisé, éventuelle réadaptation et autonomie à vérifier.</t>
+  </si>
+  <si>
+    <t>avc-orientation-apa-post-rehabilitation-001</t>
+  </si>
+  <si>
+    <t>Après un AVC, la HAS préconise une APA régulière, à adapter au stade et aux séquelles évaluées. Après la phase de rééducation, discuter un programme structuré, avec supervision initiale si nécessaire ; la rééducation des déficiences et l’AP adaptée peuvent coexister. Ne pas déduire le besoin d’un niveau 2 de la seule mention d’AVC.</t>
+  </si>
+  <si>
+    <t>Phase aiguë/subaiguë/chronique, séquelles, capacités, risques cardiovasculaires et rééducation actuelle à vérifier.</t>
+  </si>
+  <si>
+    <t>has-aps-scc-07-2022</t>
+  </si>
+  <si>
+    <t>has-aps-icc-07-2022</t>
+  </si>
+  <si>
+    <t>has-aps-bpco-07-2022</t>
+  </si>
+  <si>
+    <t>has-aps-avc-09-2022</t>
   </si>
 </sst>
 </file>
@@ -6423,7 +6474,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B15">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7088,7 +7139,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B431"/>
+  <dimension ref="A1:B435"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10536,6 +10587,38 @@
         <v>2037</v>
       </c>
       <c r="B431" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2">
+      <c r="A432" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B432" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="433" spans="1:2">
+      <c r="A433" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B433" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B434" t="s">
+        <v>2005</v>
+      </c>
+    </row>
+    <row r="435" spans="1:2">
+      <c r="A435" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B435" t="s">
         <v>2005</v>
       </c>
     </row>
@@ -10925,7 +11008,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D538"/>
+  <dimension ref="A1:D542"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17558,6 +17641,50 @@
         <v>1968</v>
       </c>
     </row>
+    <row r="539" spans="1:4">
+      <c r="A539" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B539" t="s">
+        <v>403</v>
+      </c>
+      <c r="C539" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="540" spans="1:4">
+      <c r="A540" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B540" t="s">
+        <v>403</v>
+      </c>
+      <c r="C540" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="541" spans="1:4">
+      <c r="A541" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B541" t="s">
+        <v>403</v>
+      </c>
+      <c r="C541" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="542" spans="1:4">
+      <c r="A542" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B542" t="s">
+        <v>403</v>
+      </c>
+      <c r="C542" t="s">
+        <v>1968</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17565,7 +17692,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I512"/>
+  <dimension ref="A1:I516"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30498,6 +30625,110 @@
       </c>
       <c r="I512" t="s">
         <v>2027</v>
+      </c>
+    </row>
+    <row r="513" spans="1:9">
+      <c r="A513" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B513" t="s">
+        <v>2046</v>
+      </c>
+      <c r="D513" t="s">
+        <v>55</v>
+      </c>
+      <c r="E513" t="s">
+        <v>2047</v>
+      </c>
+      <c r="F513" t="s">
+        <v>40</v>
+      </c>
+      <c r="G513" t="s">
+        <v>41</v>
+      </c>
+      <c r="H513">
+        <v>1</v>
+      </c>
+      <c r="I513" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="514" spans="1:9">
+      <c r="A514" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B514" t="s">
+        <v>2050</v>
+      </c>
+      <c r="D514" t="s">
+        <v>55</v>
+      </c>
+      <c r="E514" t="s">
+        <v>2051</v>
+      </c>
+      <c r="F514" t="s">
+        <v>40</v>
+      </c>
+      <c r="G514" t="s">
+        <v>41</v>
+      </c>
+      <c r="H514">
+        <v>1</v>
+      </c>
+      <c r="I514" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="515" spans="1:9">
+      <c r="A515" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B515" t="s">
+        <v>2053</v>
+      </c>
+      <c r="D515" t="s">
+        <v>55</v>
+      </c>
+      <c r="E515" t="s">
+        <v>2054</v>
+      </c>
+      <c r="F515" t="s">
+        <v>40</v>
+      </c>
+      <c r="G515" t="s">
+        <v>41</v>
+      </c>
+      <c r="H515">
+        <v>1</v>
+      </c>
+      <c r="I515" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="516" spans="1:9">
+      <c r="A516" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B516" t="s">
+        <v>2056</v>
+      </c>
+      <c r="D516" t="s">
+        <v>55</v>
+      </c>
+      <c r="E516" t="s">
+        <v>2057</v>
+      </c>
+      <c r="F516" t="s">
+        <v>40</v>
+      </c>
+      <c r="G516" t="s">
+        <v>41</v>
+      </c>
+      <c r="H516">
+        <v>1</v>
+      </c>
+      <c r="I516" t="s">
+        <v>2048</v>
       </c>
     </row>
   </sheetData>
@@ -30521,7 +30752,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C515"/>
+  <dimension ref="A1:C519"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36190,6 +36421,50 @@
         <v>232</v>
       </c>
       <c r="C515" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="516" spans="1:3">
+      <c r="A516" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B516" t="s">
+        <v>232</v>
+      </c>
+      <c r="C516" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="517" spans="1:3">
+      <c r="A517" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B517" t="s">
+        <v>232</v>
+      </c>
+      <c r="C517" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="518" spans="1:3">
+      <c r="A518" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B518" t="s">
+        <v>232</v>
+      </c>
+      <c r="C518" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="519" spans="1:3">
+      <c r="A519" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B519" t="s">
+        <v>232</v>
+      </c>
+      <c r="C519" t="s">
         <v>2007</v>
       </c>
     </row>
@@ -36208,7 +36483,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I512"/>
+  <dimension ref="A1:I516"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -43648,6 +43923,38 @@
       </c>
       <c r="B512" t="s">
         <v>1796</v>
+      </c>
+    </row>
+    <row r="513" spans="1:2">
+      <c r="A513" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B513" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="514" spans="1:2">
+      <c r="A514" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B514" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="515" spans="1:2">
+      <c r="A515" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B515" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="516" spans="1:2">
+      <c r="A516" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B516" t="s">
+        <v>869</v>
       </c>
     </row>
   </sheetData>
@@ -51804,7 +52111,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -51896,6 +52203,38 @@
       </c>
       <c r="B11" t="s">
         <v>2044</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>2045</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2058</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>2049</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2059</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>2052</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>2055</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2061</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation T1.1 - add arthrosis APA knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{034A0534-437D-472D-B49F-FB0383703C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442DE172-A293-4274-AC8F-C9BA0F8A04AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10995" uniqueCount="2070">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11014" uniqueCount="2075">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6247,6 +6247,21 @@
   </si>
   <si>
     <t>has-bpco-rehabilitation-2014</t>
+  </si>
+  <si>
+    <t>arthrose-orientation-apa-first-line-001</t>
+  </si>
+  <si>
+    <t>Arthrose périphérique : hors poussée congestive, un programme structuré d'APA constitue un traitement de première intention selon la HAS. Vérifier l'absence de poussée et apprécier séparément les besoins éventuels de rééducation.</t>
+  </si>
+  <si>
+    <t>Arthrose périphérique sélectionnée ; absence de poussée congestive et déficiences éventuelles à vérifier par le médecin.</t>
+  </si>
+  <si>
+    <t>T1.1 — repère Q2a arthrose : bénéfice APA sans orientation automatique ; condition clinique non inférée.</t>
+  </si>
+  <si>
+    <t>has-aps-arthrose-07-2022</t>
   </si>
 </sst>
 </file>
@@ -6498,7 +6513,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B23">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7163,7 +7178,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B436"/>
+  <dimension ref="A1:B437"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10652,6 +10667,14 @@
       </c>
       <c r="B436" t="s">
         <v>1996</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2">
+      <c r="A437" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1997</v>
       </c>
     </row>
   </sheetData>
@@ -11040,7 +11063,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D543"/>
+  <dimension ref="A1:D544"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17728,6 +17751,17 @@
         <v>1960</v>
       </c>
     </row>
+    <row r="544" spans="1:4">
+      <c r="A544" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B544" t="s">
+        <v>399</v>
+      </c>
+      <c r="C544" t="s">
+        <v>1960</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17735,7 +17769,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I517"/>
+  <dimension ref="A1:I518"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30798,6 +30832,32 @@
       </c>
       <c r="I517" t="s">
         <v>2067</v>
+      </c>
+    </row>
+    <row r="518" spans="1:9">
+      <c r="A518" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B518" t="s">
+        <v>2071</v>
+      </c>
+      <c r="D518" t="s">
+        <v>55</v>
+      </c>
+      <c r="E518" t="s">
+        <v>2072</v>
+      </c>
+      <c r="F518" t="s">
+        <v>40</v>
+      </c>
+      <c r="G518" t="s">
+        <v>41</v>
+      </c>
+      <c r="H518">
+        <v>1</v>
+      </c>
+      <c r="I518" t="s">
+        <v>2073</v>
       </c>
     </row>
   </sheetData>
@@ -30821,7 +30881,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C520"/>
+  <dimension ref="A1:C521"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36546,6 +36606,17 @@
       </c>
       <c r="C520" t="s">
         <v>422</v>
+      </c>
+    </row>
+    <row r="521" spans="1:3">
+      <c r="A521" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B521" t="s">
+        <v>231</v>
+      </c>
+      <c r="C521" t="s">
+        <v>1999</v>
       </c>
     </row>
   </sheetData>
@@ -36563,7 +36634,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I517"/>
+  <dimension ref="A1:I518"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -44043,6 +44114,14 @@
       </c>
       <c r="B517" t="s">
         <v>206</v>
+      </c>
+    </row>
+    <row r="518" spans="1:2">
+      <c r="A518" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B518" t="s">
+        <v>1096</v>
       </c>
     </row>
   </sheetData>
@@ -52199,7 +52278,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -52379,6 +52458,14 @@
       </c>
       <c r="B22" t="s">
         <v>2052</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>2070</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2074</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation T1.2 - add chronic low back pain APA knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{442DE172-A293-4274-AC8F-C9BA0F8A04AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA0B0B3-153C-4462-9A9D-44EC5C5C8048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11014" uniqueCount="2075">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11033" uniqueCount="2080">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6262,6 +6262,21 @@
   </si>
   <si>
     <t>has-aps-arthrose-07-2022</t>
+  </si>
+  <si>
+    <t>lombalgie-orientation-apa-chronic-001</t>
+  </si>
+  <si>
+    <t>Lombalgie commune chronique : un programme d’APA (niveau 2) peut être envisagé en présence d’une comorbidité, ou d’une lombalgie stabilisée avec déconditionnement à l’effort et retentissement biopsychosocial modéré. Vérifier ces critères ; les autres cadres d’activité physique restent possibles.</t>
+  </si>
+  <si>
+    <t>Lombalgie commune chronique sélectionnée ; chronicité, comorbidité, stabilisation, déconditionnement et retentissement biopsychosocial à vérifier par le médecin.</t>
+  </si>
+  <si>
+    <t>T1.2 — repère Q2a lombalgie chronique : programme d’APA (niveau 2) selon les conditions HAS ; non vérifiées automatiquement.</t>
+  </si>
+  <si>
+    <t>has-aps-lombalgie-commune-chronique-03-2024</t>
   </si>
 </sst>
 </file>
@@ -6513,7 +6528,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B24">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7178,7 +7193,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B437"/>
+  <dimension ref="A1:B438"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10674,6 +10689,14 @@
         <v>2070</v>
       </c>
       <c r="B437" t="s">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="438" spans="1:2">
+      <c r="A438" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B438" t="s">
         <v>1997</v>
       </c>
     </row>
@@ -11063,7 +11086,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D544"/>
+  <dimension ref="A1:D545"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17762,6 +17785,17 @@
         <v>1960</v>
       </c>
     </row>
+    <row r="545" spans="1:3">
+      <c r="A545" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B545" t="s">
+        <v>399</v>
+      </c>
+      <c r="C545" t="s">
+        <v>1960</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17769,7 +17803,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I518"/>
+  <dimension ref="A1:I519"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30858,6 +30892,32 @@
       </c>
       <c r="I518" t="s">
         <v>2073</v>
+      </c>
+    </row>
+    <row r="519" spans="1:9">
+      <c r="A519" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B519" t="s">
+        <v>2076</v>
+      </c>
+      <c r="D519" t="s">
+        <v>55</v>
+      </c>
+      <c r="E519" t="s">
+        <v>2077</v>
+      </c>
+      <c r="F519" t="s">
+        <v>40</v>
+      </c>
+      <c r="G519" t="s">
+        <v>41</v>
+      </c>
+      <c r="H519">
+        <v>1</v>
+      </c>
+      <c r="I519" t="s">
+        <v>2078</v>
       </c>
     </row>
   </sheetData>
@@ -30881,7 +30941,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C521"/>
+  <dimension ref="A1:C522"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36616,6 +36676,17 @@
         <v>231</v>
       </c>
       <c r="C521" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="522" spans="1:3">
+      <c r="A522" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B522" t="s">
+        <v>231</v>
+      </c>
+      <c r="C522" t="s">
         <v>1999</v>
       </c>
     </row>
@@ -36634,7 +36705,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I518"/>
+  <dimension ref="A1:I519"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -44122,6 +44193,14 @@
       </c>
       <c r="B518" t="s">
         <v>1096</v>
+      </c>
+    </row>
+    <row r="519" spans="1:2">
+      <c r="A519" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B519" t="s">
+        <v>1173</v>
       </c>
     </row>
   </sheetData>
@@ -52278,7 +52357,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -52466,6 +52545,14 @@
       </c>
       <c r="B23" t="s">
         <v>2074</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>2075</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2079</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation T1.3 - add axial spondyloarthritis APA knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA0B0B3-153C-4462-9A9D-44EC5C5C8048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9703BC3-16E7-4417-844C-0250DD96645E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11033" uniqueCount="2080">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11052" uniqueCount="2085">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6277,6 +6277,21 @@
   </si>
   <si>
     <t>has-aps-lombalgie-commune-chronique-03-2024</t>
+  </si>
+  <si>
+    <t>spa-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Spondyloarthrite axiale : un programme d’APA (niveau 2) peut être envisagé en cas de maladie modérément active, sous traitement de fond stable depuis plusieurs semaines, associée à une inactivité physique, une comorbidité et/ou un déconditionnement à l’effort. Vérifier ces conditions. En cas de maladie stabilisée avec facteurs de risque contrôlés, la HAS recommande une activité physique ordinaire encadrée (niveau 3) ou autonome (niveau 4).</t>
+  </si>
+  <si>
+    <t>Spondyloarthrite axiale sélectionnée ; activité modérée de la maladie, stabilité du traitement de fond, inactivité physique/comorbidité/déconditionnement et contrôle des facteurs de risque non inférés : à vérifier par le médecin.</t>
+  </si>
+  <si>
+    <t>T1.3 — repère Q2a SPA : programme d’APA (niveau 2) selon conditions HAS spécifiques ; possibilité de niveaux 3/4 en maladie stabilisée avec facteurs de risque contrôlés ; conditions non vérifiées automatiquement.</t>
+  </si>
+  <si>
+    <t>has-aps-spa-03-2024</t>
   </si>
 </sst>
 </file>
@@ -6528,7 +6543,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B25">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7193,7 +7208,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B438"/>
+  <dimension ref="A1:B439"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10697,6 +10712,14 @@
         <v>2075</v>
       </c>
       <c r="B438" t="s">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B439" t="s">
         <v>1997</v>
       </c>
     </row>
@@ -11086,7 +11109,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D545"/>
+  <dimension ref="A1:D546"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17796,6 +17819,17 @@
         <v>1960</v>
       </c>
     </row>
+    <row r="546" spans="1:3">
+      <c r="A546" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B546" t="s">
+        <v>399</v>
+      </c>
+      <c r="C546" t="s">
+        <v>1960</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17803,7 +17837,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I519"/>
+  <dimension ref="A1:I520"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30918,6 +30952,32 @@
       </c>
       <c r="I519" t="s">
         <v>2078</v>
+      </c>
+    </row>
+    <row r="520" spans="1:9">
+      <c r="A520" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B520" t="s">
+        <v>2081</v>
+      </c>
+      <c r="D520" t="s">
+        <v>55</v>
+      </c>
+      <c r="E520" t="s">
+        <v>2082</v>
+      </c>
+      <c r="F520" t="s">
+        <v>40</v>
+      </c>
+      <c r="G520" t="s">
+        <v>41</v>
+      </c>
+      <c r="H520">
+        <v>1</v>
+      </c>
+      <c r="I520" t="s">
+        <v>2083</v>
       </c>
     </row>
   </sheetData>
@@ -30941,7 +31001,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C522"/>
+  <dimension ref="A1:C523"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36687,6 +36747,17 @@
         <v>231</v>
       </c>
       <c r="C522" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="523" spans="1:3">
+      <c r="A523" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B523" t="s">
+        <v>231</v>
+      </c>
+      <c r="C523" t="s">
         <v>1999</v>
       </c>
     </row>
@@ -36705,7 +36776,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I519"/>
+  <dimension ref="A1:I520"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -44201,6 +44272,14 @@
       </c>
       <c r="B519" t="s">
         <v>1173</v>
+      </c>
+    </row>
+    <row r="520" spans="1:2">
+      <c r="A520" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B520" t="s">
+        <v>1319</v>
       </c>
     </row>
   </sheetData>
@@ -52357,7 +52436,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -52553,6 +52632,14 @@
       </c>
       <c r="B24" t="s">
         <v>2079</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2084</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation T1.4 - add oncology APA knowledge with attributed sources
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9703BC3-16E7-4417-844C-0250DD96645E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A93C3C39-65DB-4805-91B7-B097B3FE5FC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11052" uniqueCount="2085">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11077" uniqueCount="2093">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6292,6 +6292,30 @@
   </si>
   <si>
     <t>has-aps-spa-03-2024</t>
+  </si>
+  <si>
+    <t>cancer-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Cancer : l’activité physique adaptée est bénéfique pendant et après les traitements, notamment sur les capacités physiques, la fatigue et la qualité de vie. Un programme d’APA (niveau 2) peut être envisagé selon l’état clinique, les limitations fonctionnelles, le déconditionnement et les besoins d’accompagnement. Adapter la pratique aux traitements et aux précautions spécifiques, en lien avec l’équipe d’oncologie.</t>
+  </si>
+  <si>
+    <t>Cancer sélectionné ; localisation, traitements, limitations, déconditionnement et précautions non inférés : à apprécier par le médecin ; niveau 2 non automatique.</t>
+  </si>
+  <si>
+    <t>T1.4 — SOURCES DISTINCTES : HAS 2022 (bénéfice transversal AP, programme APA décrit pour sein/colorectal/prostate) ; INCa 2017 (bénéfices AP transversaux) ; AFSOS 2024 (référentiel tous cancers) ; ACSM 12e éd. 2025 (exercice supervisé/non supervisé, bénéfices et adaptation). Message de synthèse multi-sources ; ne pas attribuer sa totalité à la HAS.</t>
+  </si>
+  <si>
+    <t>has-aps-cancers-07-2022</t>
+  </si>
+  <si>
+    <t>inca-benefices-ap-cancer-03-2017</t>
+  </si>
+  <si>
+    <t>afsos-activite-physique-cancer-05-2024</t>
+  </si>
+  <si>
+    <t>acsm-getp-12e-oncology-2025</t>
   </si>
 </sst>
 </file>
@@ -6543,7 +6567,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B29">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7208,7 +7232,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B439"/>
+  <dimension ref="A1:B440"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10720,6 +10744,14 @@
         <v>2080</v>
       </c>
       <c r="B439" t="s">
+        <v>1997</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B440" t="s">
         <v>1997</v>
       </c>
     </row>
@@ -11109,7 +11141,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D546"/>
+  <dimension ref="A1:D547"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17830,6 +17862,17 @@
         <v>1960</v>
       </c>
     </row>
+    <row r="547" spans="1:3">
+      <c r="A547" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B547" t="s">
+        <v>399</v>
+      </c>
+      <c r="C547" t="s">
+        <v>1960</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17837,7 +17880,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I520"/>
+  <dimension ref="A1:I521"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -30978,6 +31021,32 @@
       </c>
       <c r="I520" t="s">
         <v>2083</v>
+      </c>
+    </row>
+    <row r="521" spans="1:9">
+      <c r="A521" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B521" t="s">
+        <v>2086</v>
+      </c>
+      <c r="D521" t="s">
+        <v>55</v>
+      </c>
+      <c r="E521" t="s">
+        <v>2087</v>
+      </c>
+      <c r="F521" t="s">
+        <v>40</v>
+      </c>
+      <c r="G521" t="s">
+        <v>41</v>
+      </c>
+      <c r="H521">
+        <v>1</v>
+      </c>
+      <c r="I521" t="s">
+        <v>2088</v>
       </c>
     </row>
   </sheetData>
@@ -31001,7 +31070,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C523"/>
+  <dimension ref="A1:C524"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36758,6 +36827,17 @@
         <v>231</v>
       </c>
       <c r="C523" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="524" spans="1:3">
+      <c r="A524" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B524" t="s">
+        <v>231</v>
+      </c>
+      <c r="C524" t="s">
         <v>1999</v>
       </c>
     </row>
@@ -36776,7 +36856,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I520"/>
+  <dimension ref="A1:I521"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -44280,6 +44360,14 @@
       </c>
       <c r="B520" t="s">
         <v>1319</v>
+      </c>
+    </row>
+    <row r="521" spans="1:2">
+      <c r="A521" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B521" t="s">
+        <v>1502</v>
       </c>
     </row>
   </sheetData>
@@ -52436,7 +52524,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -52640,6 +52728,38 @@
       </c>
       <c r="B25" t="s">
         <v>2084</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2089</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2090</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>2085</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2092</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Orientation T1.6 - add rheumatoid arthritis APA knowledge
</commit_message>
<xml_diff>
--- a/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
+++ b/data/clinical-knowledge/PAP_Connaissances_Cliniques_Tableur_Maitre_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\3002577\Documents\DEV\PAP\PAP-Plateforme-dev\data\clinical-knowledge\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE21FE7-E8E2-4C7E-A713-FCF7364DC2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{876F527C-1803-45B3-AB89-92F24042813F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12495" yWindow="165" windowWidth="12705" windowHeight="14865" firstSheet="11" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11098" uniqueCount="2098">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11117" uniqueCount="2103">
   <si>
     <t>PAP — Tableur maître des connaissances cliniques (prototype 7A-2E)</t>
   </si>
@@ -6331,6 +6331,21 @@
   </si>
   <si>
     <t>has-aps-sep-03-2024</t>
+  </si>
+  <si>
+    <t>pr-orientation-apa-program-001</t>
+  </si>
+  <si>
+    <t>Polyarthrite rhumatoïde : lorsque la maladie est stabilisée sous traitement, la HAS prévoit un programme d’APA (niveau 2) ou une activité encadrée (niveau 3), voire autonome (niveau 4) selon les capacités. Si la PR n’est pas stabilisée, l’orientation dépend notamment de l’activité inflammatoire (DAS28), du retentissement fonctionnel (HAQ) et des comorbidités. En cas de DAS28 élevé et de HAQ important, examiner prioritairement une rééducation (niveau 1). Lorsque ces critères sont moins marqués et en l’absence de pathologie cardiovasculaire, un programme d’APA (niveau 2) peut être envisagé, éventuellement associé à une kinésithérapie ciblée.</t>
+  </si>
+  <si>
+    <t>PR sélectionnée ; stabilité sous traitement, DAS28, HAQ, pathologie cardiovasculaire associée et déficit(s) localisé(s) non inférés : vérifier cliniquement ; ne jamais sélectionner de niveau automatiquement.</t>
+  </si>
+  <si>
+    <t>T1.6 — source HAS 28/03/2024 : PR stabilisée niveau 2/3/4 selon capacités ; PR non stabilisée DAS28 élevé/HAQ important rééducation initiale ; si critères moins importants et sans pathologie CV, APA niveau 2 envisageable. Aucun seuil automatique DAS28/HAQ ; condition cardiovasculaire limitée à la branche PR non stabilisée, ne vaut pas CI générale APA. Repère Q1 et arthroplastie existants conservés.</t>
+  </si>
+  <si>
+    <t>has-aps-pr-03-2024</t>
   </si>
 </sst>
 </file>
@@ -6582,7 +6597,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="EvidenceRefsTable" displayName="EvidenceRefsTable" ref="A1:B32">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="knowledgeItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="evidenceSourceId"/>
@@ -7247,7 +7262,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:B441"/>
+  <dimension ref="A1:B442"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -10775,6 +10790,14 @@
         <v>2093</v>
       </c>
       <c r="B441" t="s">
+        <v>1996</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2">
+      <c r="A442" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B442" t="s">
         <v>1996</v>
       </c>
     </row>
@@ -11164,7 +11187,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB74CC3-C58D-4443-B541-7C7D63A5B353}">
-  <dimension ref="A1:D548"/>
+  <dimension ref="A1:D549"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -17907,6 +17930,17 @@
         <v>1959</v>
       </c>
     </row>
+    <row r="549" spans="1:3">
+      <c r="A549" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B549" t="s">
+        <v>399</v>
+      </c>
+      <c r="C549" t="s">
+        <v>1959</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17914,7 +17948,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I522"/>
+  <dimension ref="A1:I523"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -31107,6 +31141,32 @@
       </c>
       <c r="I522" t="s">
         <v>2096</v>
+      </c>
+    </row>
+    <row r="523" spans="1:9">
+      <c r="A523" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B523" t="s">
+        <v>2099</v>
+      </c>
+      <c r="D523" t="s">
+        <v>55</v>
+      </c>
+      <c r="E523" t="s">
+        <v>2100</v>
+      </c>
+      <c r="F523" t="s">
+        <v>40</v>
+      </c>
+      <c r="G523" t="s">
+        <v>41</v>
+      </c>
+      <c r="H523">
+        <v>1</v>
+      </c>
+      <c r="I523" t="s">
+        <v>2101</v>
       </c>
     </row>
   </sheetData>
@@ -31130,7 +31190,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C525"/>
+  <dimension ref="A1:C526"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -36909,6 +36969,17 @@
         <v>231</v>
       </c>
       <c r="C525" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="526" spans="1:3">
+      <c r="A526" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B526" t="s">
+        <v>231</v>
+      </c>
+      <c r="C526" t="s">
         <v>1998</v>
       </c>
     </row>
@@ -36927,7 +36998,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I522"/>
+  <dimension ref="A1:I523"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -44447,6 +44518,14 @@
       </c>
       <c r="B522" t="s">
         <v>1033</v>
+      </c>
+    </row>
+    <row r="523" spans="1:2">
+      <c r="A523" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B523" t="s">
+        <v>1238</v>
       </c>
     </row>
   </sheetData>
@@ -52603,7 +52682,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="38" customWidth="1"/>
@@ -52855,6 +52934,14 @@
       </c>
       <c r="B31" t="s">
         <v>2097</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B32" t="s">
+        <v>2102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>